<commit_message>
docs: add guide for obtaining Shopify Admin API access token via OAuth
</commit_message>
<xml_diff>
--- a/features/bulk-update/Matrixify-ImportProducts-Demo.xlsx
+++ b/features/bulk-update/Matrixify-ImportProducts-Demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Nube\Github\ShopifyOps\features\bulk-update\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ABF0064-16F6-4E55-BF99-CCA961922A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDAF0CE-02A3-4DCA-8317-1315F828C740}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="92">
   <si>
     <t>Handle</t>
   </si>
@@ -357,7 +357,7 @@
     <t>test-product</t>
   </si>
   <si>
-    <t>Natural Honey test</t>
+    <t>other</t>
   </si>
 </sst>
 </file>
@@ -793,41 +793,41 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BL2"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" outlineLevelCol="6" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.625" style="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.375" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.375" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.125" style="8" customWidth="1"/>
-    <col min="5" max="5" width="14.875" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.375" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.375" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.125" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.375" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.875" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.125" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.125" style="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.875" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="65.875" style="8" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.875" style="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.125" style="8" customWidth="1"/>
-    <col min="20" max="20" width="69.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.375" style="8" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.375" style="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.875" style="8" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.375" style="8" hidden="1" customWidth="1" outlineLevel="6"/>
+    <col min="4" max="4" width="26.125" style="8" hidden="1" customWidth="1" outlineLevel="6"/>
+    <col min="5" max="5" width="14.875" style="8" hidden="1" customWidth="1" outlineLevel="6"/>
+    <col min="6" max="6" width="10.375" style="8" hidden="1" customWidth="1" outlineLevel="6"/>
+    <col min="7" max="7" width="27.375" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="8" max="8" width="15.125" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="9" max="9" width="8.375" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="10" max="10" width="10" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="11" max="11" width="23.875" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="12" max="12" width="16" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="13" max="13" width="15" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="14" max="14" width="9.125" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="15" max="15" width="17.125" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="16" max="16" width="20.875" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="17" max="17" width="65.875" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="18" max="18" width="18.875" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="19" max="19" width="18.125" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="20" max="20" width="69.5" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="21" max="21" width="16.375" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="22" max="22" width="14.375" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="23" max="23" width="13.875" style="8" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="24" max="24" width="9.625" style="8" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="25" max="25" width="17.125" style="8" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="13.875" style="8" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="20.375" style="8" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="13.875" style="8" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="29.625" style="8" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.875" style="8" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="23" style="8" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="29.125" style="8" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="15.125" style="8" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="13.875" style="8" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="29.625" style="8" hidden="1" customWidth="1"/>
+    <col min="30" max="30" width="13.875" style="8" hidden="1" customWidth="1"/>
+    <col min="31" max="31" width="23" style="8" hidden="1" customWidth="1"/>
+    <col min="32" max="32" width="29.125" style="8" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="15.125" style="8" hidden="1" customWidth="1"/>
     <col min="34" max="34" width="11.625" style="8" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="15.125" style="8" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="39.375" style="8" bestFit="1" customWidth="1"/>
@@ -1061,129 +1061,16 @@
       <c r="B2" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="V2" s="9"/>
+      <c r="AG2" s="9"/>
+      <c r="AH2" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="D2" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="I2" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="J2" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="K2" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="L2" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="N2" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="T2" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="U2" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="V2" s="9">
-        <v>1</v>
-      </c>
-      <c r="W2" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="Y2" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="Z2" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="AA2" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="AB2" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="AC2" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="AF2" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AG2" s="9">
-        <v>1</v>
-      </c>
-      <c r="AI2" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="AJ2" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="AK2" s="8">
-        <v>350</v>
-      </c>
-      <c r="AL2" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="AM2" s="10">
-        <v>5</v>
-      </c>
-      <c r="AN2" s="10">
-        <v>6</v>
-      </c>
-      <c r="AO2" s="10">
-        <v>3</v>
-      </c>
-      <c r="AP2" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AQ2" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="AR2" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="AS2" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="AT2" s="8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AU2" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="AV2" s="9">
-        <v>101</v>
-      </c>
-      <c r="AW2" s="9">
-        <v>0</v>
-      </c>
-      <c r="AX2" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="AY2" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="BA2" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="BB2" s="8" t="s">
-        <v>89</v>
-      </c>
+      <c r="AM2" s="10"/>
+      <c r="AN2" s="10"/>
+      <c r="AO2" s="10"/>
+      <c r="AV2" s="9"/>
+      <c r="AW2" s="9"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>